<commit_message>
Hogar de Refugio: evacuación y señalización según los planos, SS.HH. mujeres y observaciones subsanadas y pendientes
Barrido completo de símbolos del plano de señalización; las señales de SS.HH. mixto pasan a SS.HH. mujeres
(hogar solo para mujeres); documento de observaciones subsanadas en los documentos y pendientes en los planos
y en el metrado de arquitectura.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
@@ -16,13 +16,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEÑALES" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMEN'!$A$1:$D$30</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'METRADO'!$A$1:$R$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMEN'!$A$1:$D$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'METRADO'!$A$1:$R$40</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'ZONAS DE EVACUACIÓN'!$A$1:$I$27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'RUTAS DE EVACUACIÓN'!$A$1:$F$99</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'LEYENDA'!$A$1:$G$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'POBLACIÓN'!$A$1:$D$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'SEÑALES'!$A$1:$G$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'SEÑALES'!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -650,7 +650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MIXTO CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJERES CON BRAILLE</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJER CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
+          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -1074,49 +1074,49 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>01.04.05</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>01.05</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>01.05.01</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D26" s="11">
-        <f>'METRADO'!O26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>01.05</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
+      <c r="D27" s="11">
+        <f>'METRADO'!O27</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>01.05.01</t>
+          <t>01.05.02</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -1132,12 +1132,12 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>01.05.02</t>
+          <t>01.05.03</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
+          <t>DETECTOR DE HUMO</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -1147,27 +1147,6 @@
       </c>
       <c r="D29" s="11">
         <f>'METRADO'!O29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>01.05.03</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>DETECTOR DE HUMO</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="D30" s="11">
-        <f>'METRADO'!O30</f>
         <v/>
       </c>
     </row>
@@ -1192,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2127,7 +2106,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MIXTO CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJERES CON BRAILLE</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -2136,11 +2115,13 @@
         </is>
       </c>
       <c r="D23" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" s="14" t="n"/>
       <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
+      <c r="G23" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="H23" s="14" t="n"/>
       <c r="I23" s="14" t="n">
         <v>3</v>
@@ -2151,7 +2132,9 @@
       <c r="K23" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="L23" s="14" t="n"/>
+      <c r="L23" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="M23" s="14" t="n">
         <v>1</v>
       </c>
@@ -2161,7 +2144,7 @@
         <v/>
       </c>
       <c r="P23" s="14" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="Q23" s="16">
         <f>O23-P23</f>
@@ -2169,7 +2152,7 @@
       </c>
       <c r="R23" s="17" t="inlineStr">
         <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 20</t>
+          <t>Planta de SE-S-02: símbolos dibujados (3 de mujeres + 20 de "mixto", que en un hogar solo para mujeres son de mujeres); leyenda: 3</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2164,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJER CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -2231,7 +2214,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
+          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -2239,29 +2222,25 @@
           <t>und</t>
         </is>
       </c>
-      <c r="D25" s="14" t="n">
-        <v>1</v>
-      </c>
+      <c r="D25" s="14" t="n"/>
       <c r="E25" s="14" t="n"/>
       <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n">
-        <v>1</v>
-      </c>
+      <c r="G25" s="14" t="n"/>
       <c r="H25" s="14" t="n"/>
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="n"/>
       <c r="K25" s="14" t="n"/>
-      <c r="L25" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M25" s="14" t="n"/>
+      <c r="L25" s="14" t="n"/>
+      <c r="M25" s="14" t="n">
+        <v>4</v>
+      </c>
       <c r="N25" s="14" t="n"/>
       <c r="O25" s="15">
         <f>SUM(D25:N25)</f>
         <v/>
       </c>
       <c r="P25" s="14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q25" s="16">
         <f>O25-P25</f>
@@ -2269,93 +2248,109 @@
       </c>
       <c r="R25" s="17" t="inlineStr">
         <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 3</t>
+          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 0</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>04.05</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
+      <c r="O26" s="4" t="n"/>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>05.01</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="14" t="n"/>
-      <c r="K26" s="14" t="n"/>
-      <c r="L26" s="14" t="n"/>
-      <c r="M26" s="14" t="n">
+      <c r="D27" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="N26" s="14" t="n"/>
-      <c r="O26" s="15">
-        <f>SUM(D26:N26)</f>
-        <v/>
-      </c>
-      <c r="P26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="16">
-        <f>O26-P26</f>
-        <v/>
-      </c>
-      <c r="R26" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="n"/>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="n"/>
-      <c r="J27" s="4" t="n"/>
-      <c r="K27" s="4" t="n"/>
-      <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4" t="n"/>
-      <c r="P27" s="4" t="n"/>
-      <c r="Q27" s="4" t="n"/>
-      <c r="R27" s="4" t="n"/>
+      <c r="F27" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J27" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="14" t="n"/>
+      <c r="N27" s="14" t="n"/>
+      <c r="O27" s="15">
+        <f>SUM(D27:N27)</f>
+        <v/>
+      </c>
+      <c r="P27" s="14" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q27" s="16">
+        <f>O27-P27</f>
+        <v/>
+      </c>
+      <c r="R27" s="17" t="inlineStr">
+        <is>
+          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 44</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>05.01</t>
+          <t>05.02</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -2364,31 +2359,31 @@
         </is>
       </c>
       <c r="D28" s="14" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="J28" s="14" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="L28" s="14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="14" t="n"/>
@@ -2397,7 +2392,7 @@
         <v/>
       </c>
       <c r="P28" s="14" t="n">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="Q28" s="16">
         <f>O28-P28</f>
@@ -2405,19 +2400,19 @@
       </c>
       <c r="R28" s="17" t="inlineStr">
         <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 44</t>
+          <t>Planta de SE-S-02: símbolos dibujados (77 "LE" + 38 "A$C7A2016C2"); leyenda: 77</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>05.02</t>
+          <t>05.03</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
+          <t>DETECTOR DE HUMO</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -2426,40 +2421,42 @@
         </is>
       </c>
       <c r="D29" s="14" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E29" s="14" t="n">
         <v>2</v>
       </c>
       <c r="F29" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>20</v>
-      </c>
       <c r="H29" s="14" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I29" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J29" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="J29" s="14" t="n">
-        <v>21</v>
-      </c>
       <c r="K29" s="14" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L29" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="M29" s="14" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="M29" s="14" t="n">
+        <v>1</v>
+      </c>
       <c r="N29" s="14" t="n"/>
       <c r="O29" s="15">
         <f>SUM(D29:N29)</f>
         <v/>
       </c>
       <c r="P29" s="14" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="Q29" s="16">
         <f>O29-P29</f>
@@ -2467,185 +2464,121 @@
       </c>
       <c r="R29" s="17" t="inlineStr">
         <is>
-          <t>Planta de SE-S-02: símbolos dibujados (77 "LE" + 38 "A$C7A2016C2"); leyenda: 77</t>
+          <t>Planta de SE-S-02: símbolos dibujados; 1 copia fuera del terreno no se metra; leyenda: 68</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>05.03</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>DETECTOR DE HUMO</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="H30" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="I30" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="J30" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K30" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="M30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" s="14" t="n"/>
+      <c r="A30" s="21" t="n"/>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL DE SEÑALES Y EQUIPOS (und)</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="n"/>
+      <c r="D30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",D11:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",E11:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",F11:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",G11:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",H11:H29)</f>
+        <v/>
+      </c>
+      <c r="I30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",I11:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",J11:J29)</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",K11:K29)</f>
+        <v/>
+      </c>
+      <c r="L30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",L11:L29)</f>
+        <v/>
+      </c>
+      <c r="M30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",M11:M29)</f>
+        <v/>
+      </c>
+      <c r="N30" s="15">
+        <f>SUMIF($C$11:$C$29,"und",N11:N29)</f>
+        <v/>
+      </c>
       <c r="O30" s="15">
-        <f>SUM(D30:N30)</f>
-        <v/>
-      </c>
-      <c r="P30" s="14" t="n">
-        <v>68</v>
-      </c>
-      <c r="Q30" s="16">
-        <f>O30-P30</f>
-        <v/>
-      </c>
-      <c r="R30" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; 1 copia fuera del terreno no se metra; leyenda: 68</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="n"/>
-      <c r="B31" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL DE SEÑALES Y EQUIPOS (und)</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",D11:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",E11:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",F11:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",G11:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",H11:H30)</f>
-        <v/>
-      </c>
-      <c r="I31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",I11:I30)</f>
-        <v/>
-      </c>
-      <c r="J31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",J11:J30)</f>
-        <v/>
-      </c>
-      <c r="K31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",K11:K30)</f>
-        <v/>
-      </c>
-      <c r="L31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",L11:L30)</f>
-        <v/>
-      </c>
-      <c r="M31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",M11:M30)</f>
-        <v/>
-      </c>
-      <c r="N31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",N11:N30)</f>
-        <v/>
-      </c>
-      <c r="O31" s="15">
-        <f>SUMIF($C$11:$C$30,"und",O11:O30)</f>
-        <v/>
-      </c>
-      <c r="P31" s="21" t="n"/>
-      <c r="Q31" s="21" t="n"/>
-      <c r="R31" s="21" t="n"/>
-    </row>
-    <row r="33" ht="12" customHeight="1">
-      <c r="A33" s="23" t="inlineStr">
+        <f>SUMIF($C$11:$C$29,"und",O11:O29)</f>
+        <v/>
+      </c>
+      <c r="P30" s="21" t="n"/>
+      <c r="Q30" s="21" t="n"/>
+      <c r="R30" s="21" t="n"/>
+    </row>
+    <row r="32" ht="12" customHeight="1">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Notas:</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="26" customHeight="1">
+      <c r="A33" s="24" t="inlineStr">
+        <is>
+          <t>1. Cantidad por edificación: cada símbolo de la planta de la lámina SE-S-02 se asigna a la edificación donde está (contorno del bloque de la planta general, con 0.60 m de margen para las señales de fachada; donde los contornos se traslapan en los aleros, la edificación que lo contiene con más holgura); EXT = exteriores (garita de control, patios, estacionamientos, puntos ecológicos y circulaciones). No se metran las copias de símbolos que están fuera del terreno.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>1. Cantidad por edificación: cada símbolo de la planta de la lámina SE-S-02 se asigna a la edificación donde está (contorno del bloque de la planta general, con 0.60 m de margen para las señales de fachada; donde los contornos se traslapan en los aleros, la edificación que lo contiene con más holgura); EXT = exteriores (garita de control, patios, estacionamientos, puntos ecológicos y circulaciones). No se metran las copias de símbolos que están fuera del terreno.</t>
+          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no exporta su ubicación; se metran las 39 imágenes de igual tamaño del espacio modelo (la leyenda indica 38), con el reparto por edificación del metrado de evacuación de arquitectura, que suma lo mismo. Se instalan en los tableros y ambientes eléctricos que indica la lámina.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="24" t="inlineStr">
         <is>
-          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no exporta su ubicación; se metran las 39 imágenes de igual tamaño del espacio modelo (la leyenda indica 38), con el reparto por edificación del metrado de evacuación de arquitectura, que suma lo mismo. Se instalan en los tableros y ambientes eléctricos que indica la lámina.</t>
+          <t>3. Unidad de luces de emergencia: los bloques "LE" (77) y "A$C7A2016C2" (38) son el mismo símbolo de la leyenda (el primero contiene al segundo); se suman los dos: 115 und. La leyenda indica 77.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
       <c r="A36" s="24" t="inlineStr">
         <is>
-          <t>3. Unidad de luces de emergencia: los bloques "LE" (77) y "A$C7A2016C2" (38) son el mismo símbolo de la leyenda (el primero contiene al segundo); se suman los dos: 115 und. La leyenda indica 77.</t>
+          <t>4. Extintores: uno por cada señal de ubicación de extintor de la planta (33), PQS tipo ABC de 9 kg.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
       <c r="A37" s="24" t="inlineStr">
         <is>
-          <t>4. Extintores: uno por cada señal de ubicación de extintor de la planta (33), PQS tipo ABC de 9 kg.</t>
+          <t>5. DIFERENCIA = metrado - leyenda: las filas distintas de "conforme" son correcciones a la leyenda del plano (nota de observaciones de señalización).</t>
         </is>
       </c>
     </row>
     <row r="38" ht="26" customHeight="1">
       <c r="A38" s="24" t="inlineStr">
         <is>
-          <t>5. DIFERENCIA = metrado - leyenda: las filas distintas de "conforme" son correcciones a la leyenda del plano (nota de observaciones de señalización).</t>
+          <t>6. Unidades de luces de emergencia y detectores de humo: su conexión y circuitos son de instalaciones eléctricas.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>6. Unidades de luces de emergencia y detectores de humo: su conexión y circuitos son de instalaciones eléctricas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="24" t="inlineStr">
         <is>
           <t>7. Zonas de evacuación en caso de emergencia: las 13 de la lámina SE-E-01 (anillo pintado de 4.30 m de diámetro exterior y 0.15 m de ancho); el área sale de la hoja ZONAS DE EVACUACIÓN. La leyenda de SE-S-02 tiene la fila "zona de reuniones" en 00.</t>
         </is>
@@ -2654,15 +2587,16 @@
   </sheetData>
   <mergeCells count="28">
     <mergeCell ref="B4:R4"/>
+    <mergeCell ref="B26:R26"/>
     <mergeCell ref="P9:P10"/>
     <mergeCell ref="B7:R7"/>
     <mergeCell ref="A37:R37"/>
     <mergeCell ref="B3:R3"/>
     <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B27:R27"/>
     <mergeCell ref="B21:R21"/>
     <mergeCell ref="A33:R33"/>
     <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="A32:R32"/>
     <mergeCell ref="B2:R2"/>
     <mergeCell ref="B11:R11"/>
     <mergeCell ref="A35:R35"/>
@@ -2672,7 +2606,6 @@
     <mergeCell ref="N9:N10"/>
     <mergeCell ref="B19:R19"/>
     <mergeCell ref="A34:R34"/>
-    <mergeCell ref="A40:R40"/>
     <mergeCell ref="R9:R10"/>
     <mergeCell ref="A39:R39"/>
     <mergeCell ref="A9:A10"/>
@@ -2863,7 +2796,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>ZONA (RÓTULO DEL PLANO)</t>
+          <t>ZONA</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3268,19 +3201,19 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>E-06</t>
+          <t>E-04</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>349118.385</v>
+        <v>349102.335</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>9281998.475</v>
+        <v>9282001.359999999</v>
       </c>
       <c r="F22" s="14" t="n">
         <v>12</v>
@@ -3304,19 +3237,19 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>E-04</t>
+          <t>E-08</t>
         </is>
       </c>
       <c r="D23" s="18" t="n">
         <v>349102.335</v>
       </c>
       <c r="E23" s="18" t="n">
-        <v>9282001.359999999</v>
+        <v>9282019.671</v>
       </c>
       <c r="F23" s="14" t="n">
         <v>12</v>
@@ -3340,19 +3273,19 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13 (10)</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>E-08</t>
+          <t>E-06</t>
         </is>
       </c>
       <c r="D24" s="18" t="n">
-        <v>349102.335</v>
+        <v>349118.385</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>9282019.671</v>
+        <v>9281998.475</v>
       </c>
       <c r="F24" s="14" t="n">
         <v>12</v>
@@ -3397,7 +3330,7 @@
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="24" t="inlineStr">
         <is>
-          <t>Fuente: lámina SE-E-01 (bloques de zona de 4.30 m de diámetro con anillo de 0.15 m y rótulos "ZONA DE EVACUACIÓN EN CASO DE EMERGENCIA nn"); el número 10 está dos veces en el plano.</t>
+          <t>Fuente: lámina SE-E-01 (bloques de zona de 4.30 m de diámetro con anillo de 0.15 m y rótulos "ZONA DE EVACUACIÓN EN CASO DE EMERGENCIA nn"). La zona 13 figura en la lámina con el número 10, que está repetido.</t>
         </is>
       </c>
     </row>
@@ -6265,7 +6198,7 @@
         <v>20</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F15" s="16">
         <f>E15-D15</f>
@@ -6273,7 +6206,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Conforme.</t>
+          <t>Revisar.</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6228,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="F16" s="16">
         <f>E16-D16</f>
@@ -6303,7 +6236,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>Conforme.</t>
+          <t>Corregir la leyenda a 23 (lo dibujado).</t>
         </is>
       </c>
     </row>
@@ -7347,7 +7280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7877,7 +7810,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MIXTO CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJERES CON BRAILLE</t>
         </is>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -7902,7 +7835,7 @@
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>Identifica el servicio higiénico de uso mixto (habitaciones, tópico y vestidores).</t>
+          <t>Identifica el servicio higiénico de mujeres (habitaciones, tópico, vestidores, garita y SS.HH. de las edificaciones).</t>
         </is>
       </c>
     </row>
@@ -7914,7 +7847,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJER CON BRAILLE</t>
+          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -7939,7 +7872,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>Identifica el servicio higiénico de mujeres.</t>
+          <t>Identifica el servicio higiénico de varones.</t>
         </is>
       </c>
     </row>
@@ -7951,12 +7884,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
+          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>0.20 x 0.30 m</t>
+          <t>0.30 x 0.20 m</t>
         </is>
       </c>
       <c r="D24" s="17" t="inlineStr">
@@ -7971,175 +7904,138 @@
       </c>
       <c r="F24" s="29" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>Identifica el servicio higiénico de varones.</t>
+          <t>Identifica el punto de acopio selectivo de residuos sólidos (cuatro contenedores de colores).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="inlineStr">
-        <is>
-          <t>04.05</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C25" s="29" t="inlineStr">
-        <is>
-          <t>0.30 x 0.20 m</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="inlineStr">
-        <is>
-          <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
-        </is>
-      </c>
-      <c r="E25" s="29" t="inlineStr">
-        <is>
-          <t>1.80 m</t>
-        </is>
-      </c>
-      <c r="F25" s="29" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>05.01</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+        </is>
+      </c>
+      <c r="C26" s="29" t="inlineStr">
+        <is>
+          <t>extintor portátil de 9 kg, agente PQS multipropósito ABC</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Cilindro de acero con manómetro, manguera, soporte de pared y tarjeta de control</t>
+        </is>
+      </c>
+      <c r="E26" s="29" t="inlineStr">
+        <is>
+          <t>1.50 m (parte superior)</t>
+        </is>
+      </c>
+      <c r="F26" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>Identifica el punto de acopio selectivo de residuos sólidos (cuatro contenedores de colores).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>EQUIPOS DE PROTECCIÓN CONTRA INCENDIO Y EMERGENCIA</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>Combate fuegos de clase A, B y C en las nueve edificaciones.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>05.01</t>
+          <t>05.02</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
+          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">
         <is>
-          <t>extintor portátil de 9 kg, agente PQS multipropósito ABC</t>
+          <t>equipo de dos faros LED, autonomía mínima 90 min</t>
         </is>
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>Cilindro de acero con manómetro, manguera, soporte de pared y tarjeta de control</t>
+          <t>Equipo autónomo con batería recargable, 220 V</t>
         </is>
       </c>
       <c r="E27" s="29" t="inlineStr">
         <is>
-          <t>1.50 m (parte superior)</t>
+          <t>2.10 m</t>
         </is>
       </c>
       <c r="F27" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>Combate fuegos de clase A, B y C en las nueve edificaciones.</t>
+          <t>Ilumina las salidas, las circulaciones y los ambientes al cortarse la energía.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>05.02</t>
+          <t>05.03</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>UNIDAD DE LUCES DE EMERGENCIA</t>
+          <t>DETECTOR DE HUMO</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>equipo de dos faros LED, autonomía mínima 90 min</t>
+          <t>detector fotoeléctrico de techo</t>
         </is>
       </c>
       <c r="D28" s="17" t="inlineStr">
         <is>
-          <t>Equipo autónomo con batería recargable, 220 V</t>
+          <t>Equipo fotoeléctrico con base de montaje</t>
         </is>
       </c>
       <c r="E28" s="29" t="inlineStr">
         <is>
-          <t>2.10 m</t>
+          <t>techo</t>
         </is>
       </c>
       <c r="F28" s="29" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>TECHO</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>Ilumina las salidas, las circulaciones y los ambientes al cortarse la energía.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>05.03</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>DETECTOR DE HUMO</t>
-        </is>
-      </c>
-      <c r="C29" s="29" t="inlineStr">
-        <is>
-          <t>detector fotoeléctrico de techo</t>
-        </is>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>Equipo fotoeléctrico con base de montaje</t>
-        </is>
-      </c>
-      <c r="E29" s="29" t="inlineStr">
-        <is>
-          <t>techo</t>
-        </is>
-      </c>
-      <c r="F29" s="29" t="inlineStr">
-        <is>
-          <t>TECHO</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
         <is>
           <t>Detecta el humo en los ambientes en su etapa inicial.</t>
         </is>
@@ -8155,9 +8051,9 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="B5:G5"/>
     <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B26:G26"/>
     <mergeCell ref="B18:G18"/>
     <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B25:G25"/>
     <mergeCell ref="B6:G6"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Hogar de Refugio: señales de riesgo eléctrico ubicadas con el PDF de la lámina
Lectura del PDF A1 de señalización (39 imágenes de riesgo eléctrico por edificación) y comprobación de los
conteos del DXF con los textos del PDF; metrado, memoria, especificaciones y observaciones actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
@@ -2016,7 +2016,7 @@
       </c>
       <c r="R20" s="17" t="inlineStr">
         <is>
-          <t>Imagen pegada en el DXF (sin ubicación): 39 imágenes en el espacio modelo; reparto por edificación del metrado de evacuación de arquitectura; leyenda: 38</t>
+          <t>Planta de SE-S-02: 39 señales (imágenes pegadas, ubicadas en el PDF de la lámina); leyenda: 38</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
     <row r="34" ht="26" customHeight="1">
       <c r="A34" s="24" t="inlineStr">
         <is>
-          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no exporta su ubicación; se metran las 39 imágenes de igual tamaño del espacio modelo (la leyenda indica 38), con el reparto por edificación del metrado de evacuación de arquitectura, que suma lo mismo. Se instalan en los tableros y ambientes eléctricos que indica la lámina.</t>
+          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no guarda su ubicación; las 39 imágenes de la planta (la leyenda indica 38) se ubicaron una por una en el PDF de la lámina y se asignaron a su edificación.</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>Imagen pegada (OLE): 39 imágenes en el espacio modelo, sin ubicación.</t>
+          <t>Imagen pegada (OLE): 39 imágenes en la planta, ubicadas en el PDF de la lámina; corregir la leyenda a 39.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refugio evacuación y señalización: metrado limpio para impresión (sin cotejo de leyenda)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_EVACUACION_Y_SENALIZACION_HOGAR_REFUGIO.xlsx
@@ -11,18 +11,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METRADO" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ZONAS DE EVACUACIÓN" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUTAS DE EVACUACIÓN" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEYENDA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POBLACIÓN" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEÑALES" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POBLACIÓN" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEÑALES" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'RESUMEN'!$A$1:$D$29</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'METRADO'!$A$1:$R$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'METRADO'!$A$1:$O$38</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'ZONAS DE EVACUACIÓN'!$A$1:$I$27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'RUTAS DE EVACUACIÓN'!$A$1:$F$99</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'LEYENDA'!$A$1:$G$37</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'POBLACIÓN'!$A$1:$D$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'SEÑALES'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'POBLACIÓN'!$A$1:$D$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'SEÑALES'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,10 +28,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="+0;-0;&quot;conforme&quot;"/>
-    <numFmt numFmtId="165" formatCode="+0.00;-0.00;&quot;conforme&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -204,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -247,9 +243,6 @@
     <xf numFmtId="1" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -257,9 +250,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -274,7 +264,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -817,7 +807,7 @@
         </is>
       </c>
       <c r="D12" s="11">
-        <f>'METRADO'!O12</f>
+        <f>'METRADO'!N12</f>
         <v/>
       </c>
     </row>
@@ -838,7 +828,7 @@
         </is>
       </c>
       <c r="D13" s="11">
-        <f>'METRADO'!O13</f>
+        <f>'METRADO'!N13</f>
         <v/>
       </c>
     </row>
@@ -859,7 +849,7 @@
         </is>
       </c>
       <c r="D14" s="11">
-        <f>'METRADO'!O14</f>
+        <f>'METRADO'!N14</f>
         <v/>
       </c>
     </row>
@@ -880,7 +870,7 @@
         </is>
       </c>
       <c r="D15" s="11">
-        <f>'METRADO'!O15</f>
+        <f>'METRADO'!N15</f>
         <v/>
       </c>
     </row>
@@ -901,7 +891,7 @@
         </is>
       </c>
       <c r="D16" s="11">
-        <f>'METRADO'!O16</f>
+        <f>'METRADO'!N16</f>
         <v/>
       </c>
     </row>
@@ -936,7 +926,7 @@
         </is>
       </c>
       <c r="D18" s="11">
-        <f>'METRADO'!O18</f>
+        <f>'METRADO'!N18</f>
         <v/>
       </c>
     </row>
@@ -971,7 +961,7 @@
         </is>
       </c>
       <c r="D20" s="11">
-        <f>'METRADO'!O20</f>
+        <f>'METRADO'!N20</f>
         <v/>
       </c>
     </row>
@@ -1006,7 +996,7 @@
         </is>
       </c>
       <c r="D22" s="11">
-        <f>'METRADO'!O22</f>
+        <f>'METRADO'!N22</f>
         <v/>
       </c>
     </row>
@@ -1027,7 +1017,7 @@
         </is>
       </c>
       <c r="D23" s="11">
-        <f>'METRADO'!O23</f>
+        <f>'METRADO'!N23</f>
         <v/>
       </c>
     </row>
@@ -1048,7 +1038,7 @@
         </is>
       </c>
       <c r="D24" s="11">
-        <f>'METRADO'!O24</f>
+        <f>'METRADO'!N24</f>
         <v/>
       </c>
     </row>
@@ -1069,7 +1059,7 @@
         </is>
       </c>
       <c r="D25" s="11">
-        <f>'METRADO'!O25</f>
+        <f>'METRADO'!N25</f>
         <v/>
       </c>
     </row>
@@ -1104,7 +1094,7 @@
         </is>
       </c>
       <c r="D27" s="11">
-        <f>'METRADO'!O27</f>
+        <f>'METRADO'!N27</f>
         <v/>
       </c>
     </row>
@@ -1125,7 +1115,7 @@
         </is>
       </c>
       <c r="D28" s="11">
-        <f>'METRADO'!O28</f>
+        <f>'METRADO'!N28</f>
         <v/>
       </c>
     </row>
@@ -1146,7 +1136,7 @@
         </is>
       </c>
       <c r="D29" s="11">
-        <f>'METRADO'!O29</f>
+        <f>'METRADO'!N29</f>
         <v/>
       </c>
     </row>
@@ -1171,7 +1161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1188,10 +1178,7 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7.5" customWidth="1" min="14" max="14"/>
-    <col width="7.5" customWidth="1" min="15" max="15"/>
-    <col width="8.5" customWidth="1" min="16" max="16"/>
-    <col width="9" customWidth="1" min="17" max="17"/>
-    <col width="44" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1225,9 +1212,6 @@
       <c r="M2" s="4" t="n"/>
       <c r="N2" s="4" t="n"/>
       <c r="O2" s="4" t="n"/>
-      <c r="P2" s="4" t="n"/>
-      <c r="Q2" s="4" t="n"/>
-      <c r="R2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1253,9 +1237,6 @@
       <c r="M3" s="4" t="n"/>
       <c r="N3" s="4" t="n"/>
       <c r="O3" s="4" t="n"/>
-      <c r="P3" s="4" t="n"/>
-      <c r="Q3" s="4" t="n"/>
-      <c r="R3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1281,9 +1262,6 @@
       <c r="M4" s="4" t="n"/>
       <c r="N4" s="4" t="n"/>
       <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
-      <c r="Q4" s="4" t="n"/>
-      <c r="R4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1309,9 +1287,6 @@
       <c r="M5" s="4" t="n"/>
       <c r="N5" s="4" t="n"/>
       <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1337,9 +1312,6 @@
       <c r="M6" s="4" t="n"/>
       <c r="N6" s="4" t="n"/>
       <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
-      <c r="Q6" s="4" t="n"/>
-      <c r="R6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1365,9 +1337,6 @@
       <c r="M7" s="4" t="n"/>
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
-      <c r="P7" s="4" t="n"/>
-      <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1437,25 +1406,10 @@
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>SIN UBICAR</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>LEYENDA SE-S-02</t>
-        </is>
-      </c>
-      <c r="Q9" s="6" t="inlineStr">
-        <is>
-          <t>DIFERENCIA</t>
-        </is>
-      </c>
-      <c r="R9" s="6" t="inlineStr">
         <is>
           <t>FUENTE DE LA CANTIDAD</t>
         </is>
@@ -1517,9 +1471,6 @@
       </c>
       <c r="N10" s="12" t="n"/>
       <c r="O10" s="12" t="n"/>
-      <c r="P10" s="12" t="n"/>
-      <c r="Q10" s="12" t="n"/>
-      <c r="R10" s="12" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -1545,9 +1496,6 @@
       <c r="M11" s="4" t="n"/>
       <c r="N11" s="4" t="n"/>
       <c r="O11" s="4" t="n"/>
-      <c r="P11" s="4" t="n"/>
-      <c r="Q11" s="4" t="n"/>
-      <c r="R11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1593,21 +1541,13 @@
         <v>1</v>
       </c>
       <c r="M12" s="14" t="n"/>
-      <c r="N12" s="14" t="n"/>
-      <c r="O12" s="15">
-        <f>SUM(D12:N12)</f>
-        <v/>
-      </c>
-      <c r="P12" s="14" t="n">
-        <v>49</v>
-      </c>
-      <c r="Q12" s="16">
-        <f>O12-P12</f>
-        <v/>
-      </c>
-      <c r="R12" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 49</t>
+      <c r="N12" s="15">
+        <f>SUM(D12:M12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -1651,21 +1591,13 @@
       </c>
       <c r="L13" s="14" t="n"/>
       <c r="M13" s="14" t="n"/>
-      <c r="N13" s="14" t="n"/>
-      <c r="O13" s="15">
-        <f>SUM(D13:N13)</f>
-        <v/>
-      </c>
-      <c r="P13" s="14" t="n">
-        <v>63</v>
-      </c>
-      <c r="Q13" s="16">
-        <f>O13-P13</f>
-        <v/>
-      </c>
-      <c r="R13" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 63</t>
+      <c r="N13" s="15">
+        <f>SUM(D13:M13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -1713,21 +1645,13 @@
         <v>11</v>
       </c>
       <c r="M14" s="14" t="n"/>
-      <c r="N14" s="14" t="n"/>
-      <c r="O14" s="15">
-        <f>SUM(D14:N14)</f>
-        <v/>
-      </c>
-      <c r="P14" s="14" t="n">
-        <v>210</v>
-      </c>
-      <c r="Q14" s="16">
-        <f>O14-P14</f>
-        <v/>
-      </c>
-      <c r="R14" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 210</t>
+      <c r="N14" s="15">
+        <f>SUM(D14:M14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -1775,21 +1699,13 @@
         <v>1</v>
       </c>
       <c r="M15" s="14" t="n"/>
-      <c r="N15" s="14" t="n"/>
-      <c r="O15" s="15">
-        <f>SUM(D15:N15)</f>
-        <v/>
-      </c>
-      <c r="P15" s="14" t="n">
-        <v>55</v>
-      </c>
-      <c r="Q15" s="16">
-        <f>O15-P15</f>
-        <v/>
-      </c>
-      <c r="R15" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 55</t>
+      <c r="N15" s="15">
+        <f>SUM(D15:M15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -1809,34 +1725,26 @@
           <t>m2</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
-      <c r="F16" s="18" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="18" t="n"/>
-      <c r="I16" s="18" t="n"/>
-      <c r="J16" s="18" t="n"/>
-      <c r="K16" s="18" t="n"/>
-      <c r="L16" s="18" t="n"/>
-      <c r="M16" s="18">
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="17" t="n"/>
+      <c r="J16" s="17" t="n"/>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="17" t="n"/>
+      <c r="M16" s="17">
         <f>'ZONAS DE EVACUACIÓN'!G25</f>
         <v/>
       </c>
-      <c r="N16" s="18" t="n"/>
-      <c r="O16" s="19">
-        <f>SUM(D16:N16)</f>
-        <v/>
-      </c>
-      <c r="P16" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="20">
-        <f>O16-P16</f>
-        <v/>
-      </c>
-      <c r="R16" s="17" t="inlineStr">
-        <is>
-          <t>Lámina SE-E-01: 13 zonas de evacuación de 4.30 m de diámetro con anillo de 0.15 m (13 x 1.9556 m²); leyenda de SE-S-02: 00</t>
+      <c r="N16" s="18">
+        <f>SUM(D16:M16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-E-01: 13 zonas de evacuación (hoja ZONAS DE EVACUACIÓN)</t>
         </is>
       </c>
     </row>
@@ -1864,9 +1772,6 @@
       <c r="M17" s="4" t="n"/>
       <c r="N17" s="4" t="n"/>
       <c r="O17" s="4" t="n"/>
-      <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="4" t="n"/>
-      <c r="R17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -1912,21 +1817,13 @@
         <v>1</v>
       </c>
       <c r="M18" s="14" t="n"/>
-      <c r="N18" s="14" t="n"/>
-      <c r="O18" s="15">
-        <f>SUM(D18:N18)</f>
-        <v/>
-      </c>
-      <c r="P18" s="14" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q18" s="16">
-        <f>O18-P18</f>
-        <v/>
-      </c>
-      <c r="R18" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 44</t>
+      <c r="N18" s="15">
+        <f>SUM(D18:M18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -1954,9 +1851,6 @@
       <c r="M19" s="4" t="n"/>
       <c r="N19" s="4" t="n"/>
       <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2002,21 +1896,13 @@
         <v>1</v>
       </c>
       <c r="M20" s="14" t="n"/>
-      <c r="N20" s="14" t="n"/>
-      <c r="O20" s="15">
-        <f>SUM(D20:N20)</f>
-        <v/>
-      </c>
-      <c r="P20" s="14" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q20" s="16">
-        <f>O20-P20</f>
-        <v/>
-      </c>
-      <c r="R20" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: 39 señales (imágenes pegadas, ubicadas en el PDF de la lámina); leyenda: 38</t>
+      <c r="N20" s="15">
+        <f>SUM(D20:M20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -2044,9 +1930,6 @@
       <c r="M21" s="4" t="n"/>
       <c r="N21" s="4" t="n"/>
       <c r="O21" s="4" t="n"/>
-      <c r="P21" s="4" t="n"/>
-      <c r="Q21" s="4" t="n"/>
-      <c r="R21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -2080,21 +1963,13 @@
       <c r="K22" s="14" t="n"/>
       <c r="L22" s="14" t="n"/>
       <c r="M22" s="14" t="n"/>
-      <c r="N22" s="14" t="n"/>
-      <c r="O22" s="15">
-        <f>SUM(D22:N22)</f>
-        <v/>
-      </c>
-      <c r="P22" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q22" s="16">
-        <f>O22-P22</f>
-        <v/>
-      </c>
-      <c r="R22" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 3</t>
+      <c r="N22" s="15">
+        <f>SUM(D22:M22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -2138,21 +2013,13 @@
       <c r="M23" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="N23" s="14" t="n"/>
-      <c r="O23" s="15">
-        <f>SUM(D23:N23)</f>
-        <v/>
-      </c>
-      <c r="P23" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q23" s="16">
-        <f>O23-P23</f>
-        <v/>
-      </c>
-      <c r="R23" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados (3 de mujeres + 20 de "mixto", que en un hogar solo para mujeres son de mujeres); leyenda: 3</t>
+      <c r="N23" s="15">
+        <f>SUM(D23:M23)</f>
+        <v/>
+      </c>
+      <c r="O23" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: SS.HH. de las edificaciones, habitaciones, tópico, vestidores y garita</t>
         </is>
       </c>
     </row>
@@ -2188,21 +2055,13 @@
         <v>1</v>
       </c>
       <c r="M24" s="14" t="n"/>
-      <c r="N24" s="14" t="n"/>
-      <c r="O24" s="15">
-        <f>SUM(D24:N24)</f>
-        <v/>
-      </c>
-      <c r="P24" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q24" s="16">
-        <f>O24-P24</f>
-        <v/>
-      </c>
-      <c r="R24" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 3</t>
+      <c r="N24" s="15">
+        <f>SUM(D24:M24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -2234,21 +2093,13 @@
       <c r="M25" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="N25" s="14" t="n"/>
-      <c r="O25" s="15">
-        <f>SUM(D25:N25)</f>
-        <v/>
-      </c>
-      <c r="P25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="16">
-        <f>O25-P25</f>
-        <v/>
-      </c>
-      <c r="R25" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 0</t>
+      <c r="N25" s="15">
+        <f>SUM(D25:M25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -2276,9 +2127,6 @@
       <c r="M26" s="4" t="n"/>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
-      <c r="P26" s="4" t="n"/>
-      <c r="Q26" s="4" t="n"/>
-      <c r="R26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -2324,21 +2172,13 @@
         <v>1</v>
       </c>
       <c r="M27" s="14" t="n"/>
-      <c r="N27" s="14" t="n"/>
-      <c r="O27" s="15">
-        <f>SUM(D27:N27)</f>
-        <v/>
-      </c>
-      <c r="P27" s="14" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q27" s="16">
-        <f>O27-P27</f>
-        <v/>
-      </c>
-      <c r="R27" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; leyenda: 44</t>
+      <c r="N27" s="15">
+        <f>SUM(D27:M27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: un extintor por cada señal de ubicación de extintor</t>
         </is>
       </c>
     </row>
@@ -2386,21 +2226,13 @@
         <v>5</v>
       </c>
       <c r="M28" s="14" t="n"/>
-      <c r="N28" s="14" t="n"/>
-      <c r="O28" s="15">
-        <f>SUM(D28:N28)</f>
-        <v/>
-      </c>
-      <c r="P28" s="14" t="n">
-        <v>77</v>
-      </c>
-      <c r="Q28" s="16">
-        <f>O28-P28</f>
-        <v/>
-      </c>
-      <c r="R28" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados (77 "LE" + 38 "A$C7A2016C2"); leyenda: 77</t>
+      <c r="N28" s="15">
+        <f>SUM(D28:M28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
@@ -2450,32 +2282,24 @@
       <c r="M29" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="N29" s="14" t="n"/>
-      <c r="O29" s="15">
-        <f>SUM(D29:N29)</f>
-        <v/>
-      </c>
-      <c r="P29" s="14" t="n">
-        <v>68</v>
-      </c>
-      <c r="Q29" s="16">
-        <f>O29-P29</f>
-        <v/>
-      </c>
-      <c r="R29" s="17" t="inlineStr">
-        <is>
-          <t>Planta de SE-S-02: símbolos dibujados; 1 copia fuera del terreno no se metra; leyenda: 68</t>
+      <c r="N29" s="15">
+        <f>SUM(D29:M29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="16" t="inlineStr">
+        <is>
+          <t>Lámina SE-S-02: señales dibujadas en la planta</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="21" t="n"/>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>TOTAL DE SEÑALES Y EQUIPOS (und)</t>
         </is>
       </c>
-      <c r="C30" s="21" t="n"/>
+      <c r="C30" s="19" t="n"/>
       <c r="D30" s="15">
         <f>SUMIF($C$11:$C$29,"und",D11:D29)</f>
         <v/>
@@ -2520,100 +2344,75 @@
         <f>SUMIF($C$11:$C$29,"und",N11:N29)</f>
         <v/>
       </c>
-      <c r="O30" s="15">
-        <f>SUMIF($C$11:$C$29,"und",O11:O29)</f>
-        <v/>
-      </c>
-      <c r="P30" s="21" t="n"/>
-      <c r="Q30" s="21" t="n"/>
-      <c r="R30" s="21" t="n"/>
+      <c r="O30" s="19" t="n"/>
     </row>
     <row r="32" ht="12" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>Notas:</t>
         </is>
       </c>
     </row>
     <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="24" t="inlineStr">
-        <is>
-          <t>1. Cantidad por edificación: cada símbolo de la planta de la lámina SE-S-02 se asigna a la edificación donde está (contorno del bloque de la planta general, con 0.60 m de margen para las señales de fachada; donde los contornos se traslapan en los aleros, la edificación que lo contiene con más holgura); EXT = exteriores (garita de control, patios, estacionamientos, puntos ecológicos y circulaciones). No se metran las copias de símbolos que están fuera del terreno.</t>
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>1. Cantidad por edificación: cada señal y equipo de la planta de la lámina SE-S-02 se asigna a la edificación donde está instalado; EXT = exteriores (garita de control, patios, estacionamientos, puntos ecológicos y circulaciones).</t>
         </is>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>2. Atención riesgo eléctrico: en el DXF es una imagen pegada (OLE) que no guarda su ubicación; las 39 imágenes de la planta (la leyenda indica 38) se ubicaron una por una en el PDF de la lámina y se asignaron a su edificación.</t>
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>2. Señal de atención riesgo eléctrico: en los tableros y equipos eléctricos de cada edificación.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="24" t="inlineStr">
-        <is>
-          <t>3. Unidad de luces de emergencia: los bloques "LE" (77) y "A$C7A2016C2" (38) son el mismo símbolo de la leyenda (el primero contiene al segundo); se suman los dos: 115 und. La leyenda indica 77.</t>
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>3. Extintores: uno por cada señal de ubicación de extintor de la planta, PQS tipo ABC de 9 kg.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="24" t="inlineStr">
-        <is>
-          <t>4. Extintores: uno por cada señal de ubicación de extintor de la planta (33), PQS tipo ABC de 9 kg.</t>
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>4. Unidades de luces de emergencia y detectores de humo: su conexión y circuitos son de instalaciones eléctricas.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="24" t="inlineStr">
-        <is>
-          <t>5. DIFERENCIA = metrado - leyenda: las filas distintas de "conforme" son correcciones a la leyenda del plano (nota de observaciones de señalización).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="24" t="inlineStr">
-        <is>
-          <t>6. Unidades de luces de emergencia y detectores de humo: su conexión y circuitos son de instalaciones eléctricas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="24" t="inlineStr">
-        <is>
-          <t>7. Zonas de evacuación en caso de emergencia: las 13 de la lámina SE-E-01 (anillo pintado de 4.30 m de diámetro exterior y 0.15 m de ancho); el área sale de la hoja ZONAS DE EVACUACIÓN. La leyenda de SE-S-02 tiene la fila "zona de reuniones" en 00.</t>
+      <c r="A37" s="22" t="inlineStr">
+        <is>
+          <t>5. Zonas de evacuación en caso de emergencia: las de la lámina SE-E-01 (anillo pintado de 4.30 m de diámetro exterior y 0.15 m de ancho); el área sale de la hoja ZONAS DE EVACUACIÓN.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="B4:R4"/>
-    <mergeCell ref="B26:R26"/>
-    <mergeCell ref="P9:P10"/>
-    <mergeCell ref="B7:R7"/>
-    <mergeCell ref="A37:R37"/>
-    <mergeCell ref="B3:R3"/>
+  <mergeCells count="23">
+    <mergeCell ref="B26:O26"/>
+    <mergeCell ref="B4:O4"/>
+    <mergeCell ref="B7:O7"/>
+    <mergeCell ref="A37:O37"/>
+    <mergeCell ref="B3:O3"/>
     <mergeCell ref="C9:C10"/>
-    <mergeCell ref="B21:R21"/>
-    <mergeCell ref="A33:R33"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="A32:R32"/>
-    <mergeCell ref="B2:R2"/>
-    <mergeCell ref="B11:R11"/>
-    <mergeCell ref="A35:R35"/>
+    <mergeCell ref="B21:O21"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="A33:O33"/>
+    <mergeCell ref="B11:O11"/>
+    <mergeCell ref="A32:O32"/>
+    <mergeCell ref="B17:O17"/>
+    <mergeCell ref="A35:O35"/>
     <mergeCell ref="B9:B10"/>
-    <mergeCell ref="B17:R17"/>
-    <mergeCell ref="A38:R38"/>
     <mergeCell ref="N9:N10"/>
-    <mergeCell ref="B19:R19"/>
-    <mergeCell ref="A34:R34"/>
-    <mergeCell ref="R9:R10"/>
-    <mergeCell ref="A39:R39"/>
+    <mergeCell ref="B19:O19"/>
+    <mergeCell ref="A34:O34"/>
     <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B6:O6"/>
+    <mergeCell ref="A36:O36"/>
     <mergeCell ref="O9:O10"/>
-    <mergeCell ref="B6:R6"/>
-    <mergeCell ref="A36:R36"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="B5:R5"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="B5:O5"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2767,7 +2566,7 @@
           <t>Radio exterior (m)</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="17" t="n">
         <v>2.15</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2775,7 +2574,7 @@
           <t>Radio interior (m)</t>
         </is>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="17" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2783,7 +2582,7 @@
           <t>Ancho de línea (m)</t>
         </is>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <f>B9-D9</f>
         <v/>
       </c>
@@ -2849,24 +2648,24 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="17" t="n">
         <v>349128.471</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="17" t="n">
         <v>9281929.549000001</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G12" s="25">
+      <c r="G12" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H12" s="18">
+      <c r="H12" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I12" s="18">
+      <c r="I12" s="17">
         <f>H12/F12</f>
         <v/>
       </c>
@@ -2885,24 +2684,24 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="17" t="n">
         <v>349127.685</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="17" t="n">
         <v>9281951.586999999</v>
       </c>
       <c r="F13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G13" s="25">
+      <c r="G13" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H13" s="18">
+      <c r="H13" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I13" s="18">
+      <c r="I13" s="17">
         <f>H13/F13</f>
         <v/>
       </c>
@@ -2921,24 +2720,24 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="17" t="n">
         <v>349155.693</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="17" t="n">
         <v>9281949.651000001</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H14" s="18">
+      <c r="H14" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="17">
         <f>H14/F14</f>
         <v/>
       </c>
@@ -2957,24 +2756,24 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="17" t="n">
         <v>349120.395</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="17" t="n">
         <v>9281961.002</v>
       </c>
       <c r="F15" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H15" s="18">
+      <c r="H15" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I15" s="18">
+      <c r="I15" s="17">
         <f>H15/F15</f>
         <v/>
       </c>
@@ -2993,24 +2792,24 @@
           <t>E-02</t>
         </is>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="17" t="n">
         <v>349127.913</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="17" t="n">
         <v>9281959.794</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H16" s="18">
+      <c r="H16" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I16" s="18">
+      <c r="I16" s="17">
         <f>H16/F16</f>
         <v/>
       </c>
@@ -3029,24 +2828,24 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="17" t="n">
         <v>349117.799</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="17" t="n">
         <v>9281976.48</v>
       </c>
       <c r="F17" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G17" s="25">
+      <c r="G17" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H17" s="18">
+      <c r="H17" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I17" s="18">
+      <c r="I17" s="17">
         <f>H17/F17</f>
         <v/>
       </c>
@@ -3065,24 +2864,24 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="17" t="n">
         <v>349124.758</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="17" t="n">
         <v>9281968.23</v>
       </c>
       <c r="F18" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="17">
         <f>H18/F18</f>
         <v/>
       </c>
@@ -3101,24 +2900,24 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="17" t="n">
         <v>349156.666</v>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="17" t="n">
         <v>9281983.984999999</v>
       </c>
       <c r="F19" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="G19" s="25">
+      <c r="G19" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <f>H19/F19</f>
         <v/>
       </c>
@@ -3137,24 +2936,24 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="17" t="n">
         <v>349135.346</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="17" t="n">
         <v>9282013.325999999</v>
       </c>
       <c r="F20" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G20" s="25">
+      <c r="G20" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="17">
         <f>H20/F20</f>
         <v/>
       </c>
@@ -3173,24 +2972,24 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="17" t="n">
         <v>349118.84</v>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="17" t="n">
         <v>9282020.194</v>
       </c>
       <c r="F21" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H21" s="18">
+      <c r="H21" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I21" s="18">
+      <c r="I21" s="17">
         <f>H21/F21</f>
         <v/>
       </c>
@@ -3209,24 +3008,24 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="17" t="n">
         <v>349102.335</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="17" t="n">
         <v>9282001.359999999</v>
       </c>
       <c r="F22" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H22" s="18">
+      <c r="H22" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I22" s="18">
+      <c r="I22" s="17">
         <f>H22/F22</f>
         <v/>
       </c>
@@ -3245,24 +3044,24 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="17" t="n">
         <v>349102.335</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="17" t="n">
         <v>9282019.671</v>
       </c>
       <c r="F23" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G23" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H23" s="18">
+      <c r="H23" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I23" s="18">
+      <c r="I23" s="17">
         <f>H23/F23</f>
         <v/>
       </c>
@@ -3273,7 +3072,7 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>13 (10)</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -3281,24 +3080,24 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="17" t="n">
         <v>349118.385</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="17" t="n">
         <v>9281998.475</v>
       </c>
       <c r="F24" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="G24" s="25">
+      <c r="G24" s="23">
         <f>PI()*($B$9^2-$D$9^2)</f>
         <v/>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="17">
         <f>PI()*$D$9^2</f>
         <v/>
       </c>
-      <c r="I24" s="18">
+      <c r="I24" s="17">
         <f>H24/F24</f>
         <v/>
       </c>
@@ -3308,29 +3107,29 @@
         <f>COUNT(A12:A24)</f>
         <v/>
       </c>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="B25" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="21" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
       <c r="F25" s="15">
         <f>SUM(F12:F24)</f>
         <v/>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="18">
         <f>ROUND(SUM(G12:G24),2)</f>
         <v/>
       </c>
-      <c r="H25" s="21" t="n"/>
-      <c r="I25" s="21" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="24" t="inlineStr">
-        <is>
-          <t>Fuente: lámina SE-E-01 (bloques de zona de 4.30 m de diámetro con anillo de 0.15 m y rótulos "ZONA DE EVACUACIÓN EN CASO DE EMERGENCIA nn"). La zona 13 figura en la lámina con el número 10, que está repetido.</t>
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Fuente: lámina SE-E-01 (bloques de zona de 4.30 m de diámetro con anillo de 0.15 m y rótulos "ZONA DE EVACUACIÓN EN CASO DE EMERGENCIA nn" y aforo de cada zona).</t>
         </is>
       </c>
     </row>
@@ -3483,9 +3282,9 @@
           <t>Velocidad con niñas y niños o movilidad reducida (m/s)</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n"/>
-      <c r="C9" s="27" t="n"/>
-      <c r="D9" s="18" t="n">
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="17" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -3495,9 +3294,9 @@
           <t>Velocidad de adultos (m/s)</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n"/>
-      <c r="C10" s="27" t="n"/>
-      <c r="D10" s="18" t="n">
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3507,9 +3306,9 @@
           <t>Recorrido máximo sin rociadores - RNE A.130 (m)</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n"/>
-      <c r="C11" s="27" t="n"/>
-      <c r="D11" s="18" t="n">
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="17" t="n">
         <v>45</v>
       </c>
     </row>
@@ -3556,7 +3355,7 @@
           <t>EXT</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="17" t="n">
         <v>9.18</v>
       </c>
       <c r="D14" s="14">
@@ -3583,7 +3382,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="17" t="n">
         <v>16.04</v>
       </c>
       <c r="D15" s="14">
@@ -3610,7 +3409,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="17" t="n">
         <v>22.99</v>
       </c>
       <c r="D16" s="14">
@@ -3637,7 +3436,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="17" t="n">
         <v>25.07</v>
       </c>
       <c r="D17" s="14">
@@ -3664,7 +3463,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="17" t="n">
         <v>21.77</v>
       </c>
       <c r="D18" s="14">
@@ -3691,7 +3490,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="17" t="n">
         <v>15.57</v>
       </c>
       <c r="D19" s="14">
@@ -3718,7 +3517,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="17" t="n">
         <v>27.46</v>
       </c>
       <c r="D20" s="14">
@@ -3745,7 +3544,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n">
+      <c r="C21" s="17" t="n">
         <v>23.91</v>
       </c>
       <c r="D21" s="14">
@@ -3772,7 +3571,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n">
+      <c r="C22" s="17" t="n">
         <v>23.07</v>
       </c>
       <c r="D22" s="14">
@@ -3799,7 +3598,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n">
+      <c r="C23" s="17" t="n">
         <v>26.01</v>
       </c>
       <c r="D23" s="14">
@@ -3826,7 +3625,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="17" t="n">
         <v>24.78</v>
       </c>
       <c r="D24" s="14">
@@ -3853,7 +3652,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="17" t="n">
         <v>24.24</v>
       </c>
       <c r="D25" s="14">
@@ -3880,7 +3679,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="17" t="n">
         <v>24.97</v>
       </c>
       <c r="D26" s="14">
@@ -3907,7 +3706,7 @@
           <t>E-01</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n">
+      <c r="C27" s="17" t="n">
         <v>17.13</v>
       </c>
       <c r="D27" s="14">
@@ -3934,7 +3733,7 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="17" t="n">
         <v>26.29</v>
       </c>
       <c r="D28" s="14">
@@ -3961,7 +3760,7 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="C29" s="18" t="n">
+      <c r="C29" s="17" t="n">
         <v>25.29</v>
       </c>
       <c r="D29" s="14">
@@ -3988,7 +3787,7 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="C30" s="18" t="n">
+      <c r="C30" s="17" t="n">
         <v>16.63</v>
       </c>
       <c r="D30" s="14">
@@ -4015,7 +3814,7 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="C31" s="18" t="n">
+      <c r="C31" s="17" t="n">
         <v>18.64</v>
       </c>
       <c r="D31" s="14">
@@ -4042,7 +3841,7 @@
           <t>E-03</t>
         </is>
       </c>
-      <c r="C32" s="18" t="n">
+      <c r="C32" s="17" t="n">
         <v>17.65</v>
       </c>
       <c r="D32" s="14">
@@ -4069,7 +3868,7 @@
           <t>E-02</t>
         </is>
       </c>
-      <c r="C33" s="18" t="n">
+      <c r="C33" s="17" t="n">
         <v>22.01</v>
       </c>
       <c r="D33" s="14">
@@ -4096,7 +3895,7 @@
           <t>E-02</t>
         </is>
       </c>
-      <c r="C34" s="18" t="n">
+      <c r="C34" s="17" t="n">
         <v>17.08</v>
       </c>
       <c r="D34" s="14">
@@ -4123,7 +3922,7 @@
           <t>E-02</t>
         </is>
       </c>
-      <c r="C35" s="18" t="n">
+      <c r="C35" s="17" t="n">
         <v>17.23</v>
       </c>
       <c r="D35" s="14">
@@ -4150,7 +3949,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C36" s="18" t="n">
+      <c r="C36" s="17" t="n">
         <v>15.08</v>
       </c>
       <c r="D36" s="14">
@@ -4177,7 +3976,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C37" s="18" t="n">
+      <c r="C37" s="17" t="n">
         <v>16.79</v>
       </c>
       <c r="D37" s="14">
@@ -4204,7 +4003,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C38" s="18" t="n">
+      <c r="C38" s="17" t="n">
         <v>18.04</v>
       </c>
       <c r="D38" s="14">
@@ -4231,7 +4030,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C39" s="18" t="n">
+      <c r="C39" s="17" t="n">
         <v>20.66</v>
       </c>
       <c r="D39" s="14">
@@ -4258,7 +4057,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C40" s="18" t="n">
+      <c r="C40" s="17" t="n">
         <v>25.76</v>
       </c>
       <c r="D40" s="14">
@@ -4285,7 +4084,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C41" s="18" t="n">
+      <c r="C41" s="17" t="n">
         <v>23.25</v>
       </c>
       <c r="D41" s="14">
@@ -4312,7 +4111,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C42" s="18" t="n">
+      <c r="C42" s="17" t="n">
         <v>21.26</v>
       </c>
       <c r="D42" s="14">
@@ -4339,7 +4138,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C43" s="18" t="n">
+      <c r="C43" s="17" t="n">
         <v>16.49</v>
       </c>
       <c r="D43" s="14">
@@ -4366,7 +4165,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C44" s="18" t="n">
+      <c r="C44" s="17" t="n">
         <v>16.49</v>
       </c>
       <c r="D44" s="14">
@@ -4393,7 +4192,7 @@
           <t>E-05</t>
         </is>
       </c>
-      <c r="C45" s="18" t="n">
+      <c r="C45" s="17" t="n">
         <v>12.49</v>
       </c>
       <c r="D45" s="14">
@@ -4420,7 +4219,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C46" s="18" t="n">
+      <c r="C46" s="17" t="n">
         <v>17.11</v>
       </c>
       <c r="D46" s="14">
@@ -4447,7 +4246,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C47" s="18" t="n">
+      <c r="C47" s="17" t="n">
         <v>14.07</v>
       </c>
       <c r="D47" s="14">
@@ -4474,7 +4273,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C48" s="18" t="n">
+      <c r="C48" s="17" t="n">
         <v>22.36</v>
       </c>
       <c r="D48" s="14">
@@ -4501,7 +4300,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C49" s="18" t="n">
+      <c r="C49" s="17" t="n">
         <v>18.63</v>
       </c>
       <c r="D49" s="14">
@@ -4528,7 +4327,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C50" s="18" t="n">
+      <c r="C50" s="17" t="n">
         <v>21.25</v>
       </c>
       <c r="D50" s="14">
@@ -4555,7 +4354,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C51" s="18" t="n">
+      <c r="C51" s="17" t="n">
         <v>16.11</v>
       </c>
       <c r="D51" s="14">
@@ -4582,7 +4381,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C52" s="18" t="n">
+      <c r="C52" s="17" t="n">
         <v>27.05</v>
       </c>
       <c r="D52" s="14">
@@ -4609,7 +4408,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C53" s="18" t="n">
+      <c r="C53" s="17" t="n">
         <v>32.72</v>
       </c>
       <c r="D53" s="14">
@@ -4636,7 +4435,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C54" s="18" t="n">
+      <c r="C54" s="17" t="n">
         <v>11.94</v>
       </c>
       <c r="D54" s="14">
@@ -4663,7 +4462,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C55" s="18" t="n">
+      <c r="C55" s="17" t="n">
         <v>7.86</v>
       </c>
       <c r="D55" s="14">
@@ -4690,7 +4489,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C56" s="18" t="n">
+      <c r="C56" s="17" t="n">
         <v>6.35</v>
       </c>
       <c r="D56" s="14">
@@ -4717,7 +4516,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C57" s="18" t="n">
+      <c r="C57" s="17" t="n">
         <v>10.4</v>
       </c>
       <c r="D57" s="14">
@@ -4744,7 +4543,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C58" s="18" t="n">
+      <c r="C58" s="17" t="n">
         <v>38.57</v>
       </c>
       <c r="D58" s="14">
@@ -4771,7 +4570,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C59" s="18" t="n">
+      <c r="C59" s="17" t="n">
         <v>15.38</v>
       </c>
       <c r="D59" s="14">
@@ -4798,7 +4597,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C60" s="18" t="n">
+      <c r="C60" s="17" t="n">
         <v>11.87</v>
       </c>
       <c r="D60" s="14">
@@ -4825,7 +4624,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C61" s="18" t="n">
+      <c r="C61" s="17" t="n">
         <v>28.87</v>
       </c>
       <c r="D61" s="14">
@@ -4852,7 +4651,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C62" s="18" t="n">
+      <c r="C62" s="17" t="n">
         <v>23.34</v>
       </c>
       <c r="D62" s="14">
@@ -4879,7 +4678,7 @@
           <t>E-07</t>
         </is>
       </c>
-      <c r="C63" s="18" t="n">
+      <c r="C63" s="17" t="n">
         <v>28.35</v>
       </c>
       <c r="D63" s="14">
@@ -4906,7 +4705,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C64" s="18" t="n">
+      <c r="C64" s="17" t="n">
         <v>24.98</v>
       </c>
       <c r="D64" s="14">
@@ -4933,7 +4732,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C65" s="18" t="n">
+      <c r="C65" s="17" t="n">
         <v>20.54</v>
       </c>
       <c r="D65" s="14">
@@ -4960,7 +4759,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C66" s="18" t="n">
+      <c r="C66" s="17" t="n">
         <v>25.74</v>
       </c>
       <c r="D66" s="14">
@@ -4987,7 +4786,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C67" s="18" t="n">
+      <c r="C67" s="17" t="n">
         <v>38.19</v>
       </c>
       <c r="D67" s="14">
@@ -5014,7 +4813,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C68" s="18" t="n">
+      <c r="C68" s="17" t="n">
         <v>17.27</v>
       </c>
       <c r="D68" s="14">
@@ -5041,7 +4840,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C69" s="18" t="n">
+      <c r="C69" s="17" t="n">
         <v>16.81</v>
       </c>
       <c r="D69" s="14">
@@ -5068,7 +4867,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C70" s="18" t="n">
+      <c r="C70" s="17" t="n">
         <v>12.78</v>
       </c>
       <c r="D70" s="14">
@@ -5095,7 +4894,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C71" s="18" t="n">
+      <c r="C71" s="17" t="n">
         <v>10.56</v>
       </c>
       <c r="D71" s="14">
@@ -5122,7 +4921,7 @@
           <t>E-08</t>
         </is>
       </c>
-      <c r="C72" s="18" t="n">
+      <c r="C72" s="17" t="n">
         <v>7.07</v>
       </c>
       <c r="D72" s="14">
@@ -5149,7 +4948,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C73" s="18" t="n">
+      <c r="C73" s="17" t="n">
         <v>7.07</v>
       </c>
       <c r="D73" s="14">
@@ -5176,7 +4975,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C74" s="18" t="n">
+      <c r="C74" s="17" t="n">
         <v>18.64</v>
       </c>
       <c r="D74" s="14">
@@ -5203,7 +5002,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C75" s="18" t="n">
+      <c r="C75" s="17" t="n">
         <v>20.78</v>
       </c>
       <c r="D75" s="14">
@@ -5230,7 +5029,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C76" s="18" t="n">
+      <c r="C76" s="17" t="n">
         <v>19.63</v>
       </c>
       <c r="D76" s="14">
@@ -5257,7 +5056,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C77" s="18" t="n">
+      <c r="C77" s="17" t="n">
         <v>16.15</v>
       </c>
       <c r="D77" s="14">
@@ -5284,7 +5083,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C78" s="18" t="n">
+      <c r="C78" s="17" t="n">
         <v>34.23</v>
       </c>
       <c r="D78" s="14">
@@ -5311,7 +5110,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C79" s="18" t="n">
+      <c r="C79" s="17" t="n">
         <v>34.38</v>
       </c>
       <c r="D79" s="14">
@@ -5338,7 +5137,7 @@
           <t>E-06</t>
         </is>
       </c>
-      <c r="C80" s="18" t="n">
+      <c r="C80" s="17" t="n">
         <v>31.11</v>
       </c>
       <c r="D80" s="14">
@@ -5365,7 +5164,7 @@
           <t>EXT</t>
         </is>
       </c>
-      <c r="C81" s="18" t="n">
+      <c r="C81" s="17" t="n">
         <v>15.77</v>
       </c>
       <c r="D81" s="14">
@@ -5392,7 +5191,7 @@
           <t>EXT</t>
         </is>
       </c>
-      <c r="C82" s="18" t="n">
+      <c r="C82" s="17" t="n">
         <v>12.58</v>
       </c>
       <c r="D82" s="14">
@@ -5419,7 +5218,7 @@
           <t>EXT</t>
         </is>
       </c>
-      <c r="C83" s="18" t="n">
+      <c r="C83" s="17" t="n">
         <v>12.58</v>
       </c>
       <c r="D83" s="14">
@@ -5446,7 +5245,7 @@
           <t>EXT</t>
         </is>
       </c>
-      <c r="C84" s="18" t="n">
+      <c r="C84" s="17" t="n">
         <v>15.77</v>
       </c>
       <c r="D84" s="14">
@@ -5473,7 +5272,7 @@
           <t>E-09</t>
         </is>
       </c>
-      <c r="C85" s="18" t="n">
+      <c r="C85" s="17" t="n">
         <v>35.75</v>
       </c>
       <c r="D85" s="14">
@@ -5500,7 +5299,7 @@
           <t>E-09</t>
         </is>
       </c>
-      <c r="C86" s="18" t="n">
+      <c r="C86" s="17" t="n">
         <v>39.67</v>
       </c>
       <c r="D86" s="14">
@@ -5527,7 +5326,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C87" s="18" t="n">
+      <c r="C87" s="17" t="n">
         <v>19.21</v>
       </c>
       <c r="D87" s="14">
@@ -5554,7 +5353,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C88" s="18" t="n">
+      <c r="C88" s="17" t="n">
         <v>16.46</v>
       </c>
       <c r="D88" s="14">
@@ -5581,7 +5380,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C89" s="18" t="n">
+      <c r="C89" s="17" t="n">
         <v>13.48</v>
       </c>
       <c r="D89" s="14">
@@ -5608,7 +5407,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C90" s="18" t="n">
+      <c r="C90" s="17" t="n">
         <v>13.13</v>
       </c>
       <c r="D90" s="14">
@@ -5635,7 +5434,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C91" s="18" t="n">
+      <c r="C91" s="17" t="n">
         <v>9.960000000000001</v>
       </c>
       <c r="D91" s="14">
@@ -5662,7 +5461,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C92" s="18" t="n">
+      <c r="C92" s="17" t="n">
         <v>7.31</v>
       </c>
       <c r="D92" s="14">
@@ -5689,7 +5488,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C93" s="18" t="n">
+      <c r="C93" s="17" t="n">
         <v>25.85</v>
       </c>
       <c r="D93" s="14">
@@ -5716,7 +5515,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C94" s="18" t="n">
+      <c r="C94" s="17" t="n">
         <v>18.31</v>
       </c>
       <c r="D94" s="14">
@@ -5743,7 +5542,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C95" s="18" t="n">
+      <c r="C95" s="17" t="n">
         <v>24.15</v>
       </c>
       <c r="D95" s="14">
@@ -5770,7 +5569,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C96" s="18" t="n">
+      <c r="C96" s="17" t="n">
         <v>21.18</v>
       </c>
       <c r="D96" s="14">
@@ -5797,7 +5596,7 @@
           <t>E-04</t>
         </is>
       </c>
-      <c r="C97" s="18" t="n">
+      <c r="C97" s="17" t="n">
         <v>17.67</v>
       </c>
       <c r="D97" s="14">
@@ -5814,7 +5613,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="28" t="inlineStr">
+      <c r="A98" s="26" t="inlineStr">
         <is>
           <t>RUTAS</t>
         </is>
@@ -5823,7 +5622,7 @@
         <f>COUNTA(A14:A97)</f>
         <v/>
       </c>
-      <c r="C98" s="19">
+      <c r="C98" s="18">
         <f>MAX(C14:C97)</f>
         <v/>
       </c>
@@ -5841,7 +5640,7 @@
       </c>
     </row>
     <row r="99" ht="26" customHeight="1">
-      <c r="A99" s="24" t="inlineStr">
+      <c r="A99" s="22" t="inlineStr">
         <is>
           <t>Fila RUTAS: cantidad de rutas, longitud y tiempos máximos y rutas que cumplen. Longitud = la rotulada en la lámina (“RUTA n - DISTANCIA”); la edificación de origen es la del punto de partida de la ruta (círculo con X en la puerta).</t>
         </is>
@@ -5872,1017 +5671,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>COTEJO DE LA LEYENDA DE LA LÁMINA SE-S-02 CON LA PLANTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>PROYECTO</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>“CREACIÓN DEL SERVICIO DE PROTECCIÓN A MUJERES VÍCTIMAS DE VIOLENCIA EN SITUACIÓN DE RIESGO DE FEMINICIDIO O PELIGRE SU INTEGRIDAD Y/O SALUD FÍSICA Y/O MENTAL EN HOGAR DE REFUGIO TEMPORAL DISTRITO DE MORALES DE LA PROVINCIA DE SAN MARTÍN DEL DEPARTAMENTO DE SAN MARTÍN”</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>CUI</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>N.° 2675514</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>ESPECIALIDAD</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>ARQUITECTURA - EVACUACIÓN Y SEÑALIZACIÓN</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>UBICACIÓN</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Distrito de Morales, provincia y departamento de San Martín</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>LÁMINAS</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>SE-E-01 Planta general de evacuación (esc. 1/150) y SE-S-02 Planta general de señalización (esc. 1/150)</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>FECHA</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>OCTUBRE 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>N.°</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>FILA DE LA LEYENDA (TEXTO DEL PLANO)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>ALTURA EN LA LEYENDA</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>CANTIDAD EN LA LEYENDA</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>DIBUJADO EN LA PLANTA</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>DIFERENCIA</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>OBSERVACIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>SALIDA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>49</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>49</v>
-      </c>
-      <c r="F10" s="16">
-        <f>E10-D10</f>
-        <v/>
-      </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>Conforme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>SEÑALES DE SERVICIOS HIGIENICOS PHD CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="16">
-        <f>E11-D11</f>
-        <v/>
-      </c>
-      <c r="G11" s="17" t="inlineStr">
-        <is>
-          <t>Conforme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>ZONA SEGURA EN CASO DE SISMO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>210</v>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>209</v>
-      </c>
-      <c r="F12" s="16">
-        <f>E12-D12</f>
-        <v/>
-      </c>
-      <c r="G12" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 209 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>AVISADOR SONORO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="16">
-        <f>E13-D13</f>
-        <v/>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>ESCALERA DE SALIDA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="16">
-        <f>E14-D14</f>
-        <v/>
-      </c>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>SEÑALES DE SERVICIOS HIGIENICOS MIXTO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="16">
-        <f>E15-D15</f>
-        <v/>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>Revisar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>SEÑALES DE SERVICIOS HIGIENICOS MUJER CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>23</v>
-      </c>
-      <c r="F16" s="16">
-        <f>E16-D16</f>
-        <v/>
-      </c>
-      <c r="G16" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 23 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>SEÑALES DE SERVICIOS HIGIENICOS VARÓN CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="16">
-        <f>E17-D17</f>
-        <v/>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>Conforme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>SEÑAL DE UBICACIÓN DE EXTINTOR PQS CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="n">
-        <v>44</v>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>33</v>
-      </c>
-      <c r="F18" s="16">
-        <f>E18-D18</f>
-        <v/>
-      </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 33 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>SEÑAL DE UBICACIÓN DE EXTINTOR CO2 CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="16">
-        <f>E19-D19</f>
-        <v/>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>SEÑAL DE UBICACIÓN DE EXTINTOR K CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="16">
-        <f>E20-D20</f>
-        <v/>
-      </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>ALARMA CONTRA INCEDIOS CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="16">
-        <f>E21-D21</f>
-        <v/>
-      </c>
-      <c r="G21" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>DETECTOR DE HUMO</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>TECHO</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>68</v>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>67</v>
-      </c>
-      <c r="F22" s="16">
-        <f>E22-D22</f>
-        <v/>
-      </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 67 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>BARRA ANTIPÁNICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>PUERTA</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="16">
-        <f>E23-D23</f>
-        <v/>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>UNIDAD DE LUCES DE EMERGENCIA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>77</v>
-      </c>
-      <c r="E24" s="14" t="n">
-        <v>115</v>
-      </c>
-      <c r="F24" s="16">
-        <f>E24-D24</f>
-        <v/>
-      </c>
-      <c r="G24" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 115 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="n">
-        <v>16</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>BOTIQUIN PRIMEROS AUXILIOS CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="16">
-        <f>E25-D25</f>
-        <v/>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>ATENCIÓN RIESGO ELECTRICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="n">
-        <v>38</v>
-      </c>
-      <c r="E26" s="14" t="n">
-        <v>39</v>
-      </c>
-      <c r="F26" s="16">
-        <f>E26-D26</f>
-        <v/>
-      </c>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>Imagen pegada (OLE): 39 imágenes en la planta, ubicadas en el PDF de la lámina; corregir la leyenda a 39.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>RIESGO DE DESCARGA ELECTRICA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="16">
-        <f>E27-D27</f>
-        <v/>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>PROHIBIDO EL INGRESO SOLO PERSONAL AUTORIZADO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="16">
-        <f>E28-D28</f>
-        <v/>
-      </c>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="n">
-        <v>20</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>SENSOR DE TEMPERATURA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>TECHO</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="16">
-        <f>E29-D29</f>
-        <v/>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>PUNTO ECOLÓGICO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="F30" s="16">
-        <f>E30-D30</f>
-        <v/>
-      </c>
-      <c r="G30" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 4 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>POZO A TIERRA CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Suelo</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="16">
-        <f>E31-D31</f>
-        <v/>
-      </c>
-      <c r="G31" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>CENTRAL DE ALARMA CONTRA INCENDIO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="16">
-        <f>E32-D32</f>
-        <v/>
-      </c>
-      <c r="G32" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>ZONA DE REUNIONES CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>EN PISO</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="14" t="n">
-        <v>25.42</v>
-      </c>
-      <c r="F33" s="16">
-        <f>E33-D33</f>
-        <v/>
-      </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>Corregir la leyenda a 25 (lo dibujado).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>LETRERO DE AFORO CON BRAILLE</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>55</v>
-      </c>
-      <c r="E34" s="14" t="n">
-        <v>55</v>
-      </c>
-      <c r="F34" s="16">
-        <f>E34-D34</f>
-        <v/>
-      </c>
-      <c r="G34" s="17" t="inlineStr">
-        <is>
-          <t>Conforme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>PANEL DE ALARMA CONTRA INCENDIO</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="16">
-        <f>E35-D35</f>
-        <v/>
-      </c>
-      <c r="G35" s="17" t="inlineStr">
-        <is>
-          <t>Sin símbolos en la planta; no se metra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>DIRECCIÓN DE EVACUACIÓN</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="D36" s="14" t="n">
-        <v>63</v>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>63</v>
-      </c>
-      <c r="F36" s="16">
-        <f>E36-D36</f>
-        <v/>
-      </c>
-      <c r="G36" s="17" t="inlineStr">
-        <is>
-          <t>Conforme.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="21" t="n"/>
-      <c r="B37" s="22" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="15">
-        <f>SUM(D10:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="15">
-        <f>SUM(E10:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="15">
-        <f>SUM(F10:F36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="21" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B6:G6"/>
-  </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
   <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7131,7 +5919,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>RESIDENTES (mujeres con sus hijas e hijos)</t>
         </is>
@@ -7140,7 +5928,7 @@
         <f>SUM(B10:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="21" t="n"/>
+      <c r="C17" s="19" t="n"/>
       <c r="D17" s="15">
         <f>SUM(D10:D16)</f>
         <v/>
@@ -7174,7 +5962,7 @@
           <t>Plazas de las habitaciones (A.030 art. 5)</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n"/>
+      <c r="C20" s="25" t="n"/>
       <c r="D20" s="14">
         <f>D17</f>
         <v/>
@@ -7191,23 +5979,23 @@
           <t>Administrativo, atención especializada, mantenimiento y vigilancia</t>
         </is>
       </c>
-      <c r="C21" s="27" t="n"/>
+      <c r="C21" s="25" t="n"/>
       <c r="D21" s="14" t="n">
         <v>62</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>Permanentes</t>
         </is>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>Residentes + personal</t>
         </is>
       </c>
-      <c r="C22" s="27" t="n"/>
+      <c r="C22" s="25" t="n"/>
       <c r="D22" s="15">
         <f>D20+D21</f>
         <v/>
@@ -7224,30 +6012,30 @@
           <t>Visitas, talleres, sala de reuniones y personal eventual</t>
         </is>
       </c>
-      <c r="C23" s="27" t="n"/>
+      <c r="C23" s="25" t="n"/>
       <c r="D23" s="14" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="inlineStr">
+      <c r="A24" s="20" t="inlineStr">
         <is>
           <t>CAPACIDAD MÁXIMA</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>Permanentes + temporales</t>
         </is>
       </c>
-      <c r="C24" s="27" t="n"/>
+      <c r="C24" s="25" t="n"/>
       <c r="D24" s="15">
         <f>D22+D23</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>Fuente: residentes = tabla de plazas de la memoria descriptiva de arquitectura (23 habitaciones); personal y temporales = memoria de evacuación de arquitectura del hogar.</t>
         </is>
@@ -7274,13 +6062,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7288,8 +6076,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -7314,7 +6101,6 @@
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
       <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -7331,7 +6117,6 @@
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -7348,7 +6133,6 @@
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
       <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -7365,7 +6149,6 @@
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -7382,7 +6165,6 @@
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -7399,7 +6181,6 @@
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -7428,11 +6209,6 @@
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>ALTURA EN LA LEYENDA</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>FUNCIÓN Y UBICACIÓN</t>
         </is>
@@ -7453,188 +6229,162 @@
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>01.01</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE SALIDA CON BRAILLE</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>0.30 x 0.20 m</t>
         </is>
       </c>
-      <c r="D11" s="17" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil fotoluminiscente impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>2.10 m</t>
         </is>
       </c>
-      <c r="F11" s="29" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Indica la puerta de salida de cada ambiente y de cada edificación hacia la circulación exterior; sobre el dintel.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>01.02</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE DIRECCIÓN DE EVACUACIÓN</t>
         </is>
       </c>
-      <c r="C12" s="29" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil fotoluminiscente impreso</t>
         </is>
       </c>
-      <c r="E12" s="29" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>2.10 m</t>
         </is>
       </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Indica con una flecha el sentido de la ruta de evacuación en pasadizos y circulaciones, hasta la salida.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>01.03</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE ZONA SEGURA EN CASO DE SISMO CON BRAILLE</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil fotoluminiscente impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F13" s="29" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Identifica los lugares de protección dentro de los ambientes (columnas y muros estructurales) durante un sismo.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>01.04</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>LETRERO DE AFORO CON BRAILLE</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>0.30 x 0.20 m</t>
         </is>
       </c>
-      <c r="D14" s="17" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E14" s="29" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>2.10 m</t>
         </is>
       </c>
-      <c r="F14" s="29" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>Indica la capacidad máxima de personas del ambiente; junto al ingreso, en el lado de la cerradura.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>01.05</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>PINTURA DE ZONA DE EVACUACIÓN EN CASO DE EMERGENCIA EN PISO (CÍRCULO DE 4.30 m, LÍNEA DE 0.15 m)</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>anillo de 4.30 m de diámetro exterior y 0.15 m de ancho</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Pintura de tránsito color amarillo sobre piso de concreto</t>
         </is>
       </c>
-      <c r="E15" s="29" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>en piso</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>EN PISO</t>
-        </is>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>Zona exterior de concentración de los ocupantes al final de las rutas de evacuación (zonas 01 a 13 de la lámina SE-E-01).</t>
         </is>
@@ -7655,40 +6405,34 @@
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>02.01</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE UBICACIÓN DE EXTINTOR PQS CON BRAILLE</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil fotoluminiscente impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E17" s="29" t="inlineStr">
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F17" s="29" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Identifica la ubicación del extintor de polvo químico seco; sobre el equipo.</t>
         </is>
@@ -7709,40 +6453,34 @@
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="29" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>03.01</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE ATENCIÓN RIESGO ELÉCTRICO CON BRAILLE</t>
         </is>
       </c>
-      <c r="C19" s="29" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E19" s="29" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>1.10 m</t>
         </is>
       </c>
-      <c r="F19" s="29" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>Advierte la presencia de tableros y equipos eléctricos; en la puerta o el frente del tablero.</t>
         </is>
@@ -7763,151 +6501,130 @@
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>04.01</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE SERVICIOS HIGIÉNICOS PARA PERSONAS CON DISCAPACIDAD CON BRAILLE</t>
         </is>
       </c>
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E21" s="29" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F21" s="29" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>Identifica el servicio higiénico accesible.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>04.02</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE SERVICIOS HIGIÉNICOS MUJERES CON BRAILLE</t>
         </is>
       </c>
-      <c r="C22" s="29" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E22" s="29" t="inlineStr">
+      <c r="E22" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F22" s="29" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Identifica el servicio higiénico de mujeres (habitaciones, tópico, vestidores, garita y SS.HH. de las edificaciones).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>04.03</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE SERVICIOS HIGIÉNICOS VARÓN CON BRAILLE</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>0.20 x 0.30 m</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E23" s="29" t="inlineStr">
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F23" s="29" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Identifica el servicio higiénico de varones.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>04.04</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>SEÑAL DE PUNTO ECOLÓGICO CON BRAILLE</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>0.30 x 0.20 m</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Lámina de PVC celtex de 3 mm con vinil adhesivo impreso y placa de acrílico con texto en braille</t>
         </is>
       </c>
-      <c r="E24" s="29" t="inlineStr">
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>1.80 m</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Identifica el punto de acopio selectivo de residuos sólidos (cuatro contenedores de colores).</t>
         </is>
@@ -7928,114 +6645,98 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>05.01</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>EXTINTOR DE POLVO QUÍMICO SECO (PQS) TIPO ABC DE 9 kg</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
         <is>
           <t>extintor portátil de 9 kg, agente PQS multipropósito ABC</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Cilindro de acero con manómetro, manguera, soporte de pared y tarjeta de control</t>
         </is>
       </c>
-      <c r="E26" s="29" t="inlineStr">
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>1.50 m (parte superior)</t>
         </is>
       </c>
-      <c r="F26" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Combate fuegos de clase A, B y C en las nueve edificaciones.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="29" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>05.02</t>
         </is>
       </c>
-      <c r="B27" s="17" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>UNIDAD DE LUCES DE EMERGENCIA</t>
         </is>
       </c>
-      <c r="C27" s="29" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
         <is>
           <t>equipo de dos faros LED, autonomía mínima 90 min</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>Equipo autónomo con batería recargable, 220 V</t>
         </is>
       </c>
-      <c r="E27" s="29" t="inlineStr">
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>2.10 m</t>
         </is>
       </c>
-      <c r="F27" s="29" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Ilumina las salidas, las circulaciones y los ambientes al cortarse la energía.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="inlineStr">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B28" s="17" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>DETECTOR DE HUMO</t>
         </is>
       </c>
-      <c r="C28" s="29" t="inlineStr">
+      <c r="C28" s="27" t="inlineStr">
         <is>
           <t>detector fotoeléctrico de techo</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>Equipo fotoeléctrico con base de montaje</t>
         </is>
       </c>
-      <c r="E28" s="29" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>techo</t>
         </is>
       </c>
-      <c r="F28" s="29" t="inlineStr">
-        <is>
-          <t>TECHO</t>
-        </is>
-      </c>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Detecta el humo en los ambientes en su etapa inicial.</t>
         </is>
@@ -8043,18 +6744,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B7:G7"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B18:F18"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>